<commit_message>
added reference and updated resource card to show title
</commit_message>
<xml_diff>
--- a/methods_navigator/data/crosswalk.xlsx
+++ b/methods_navigator/data/crosswalk.xlsx
@@ -8,23 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Scott.Coffin\Documents\Claude\Projects\Quality Manuscript\methods_navigator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50F0CD4-6CB5-4170-8F58-0688FB067D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54853E3-F5AB-4777-BF53-063D8924D940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25974" yWindow="-4008" windowWidth="34995" windowHeight="19060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Crosswalk Table" sheetId="1" r:id="rId1"/>
     <sheet name="Reviewer" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Crosswalk Table'!$A$2:$BB$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Crosswalk Table'!$A$2:$BB$189</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2653" uniqueCount="1444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2667" uniqueCount="1451">
   <si>
     <t>Reviewer Name</t>
   </si>
@@ -4575,6 +4575,27 @@
   </si>
   <si>
     <t>Review and guidance</t>
+  </si>
+  <si>
+    <t>Al-Zawaidah &amp; Waldschläger, 2026</t>
+  </si>
+  <si>
+    <t>A practical checklist for where, when, and what to measure - A systematic review of ten years of laboratory research on microplastic transport in rivers and transitional zones</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.1186/s43591-026-00190-9</t>
+  </si>
+  <si>
+    <t>Freshwater, Marine Water</t>
+  </si>
+  <si>
+    <t>Microplastic pollution in freshwater is a global concern, yet field monitoring often lacks standardization, hindering data comparability and analysis. This systematic review bridges the gap between lab findings and field sampling by analyzing 173 peer-reviewed laboratory studies on freshwater systems, published in English and identified through Web of Science up to August 2024, to extract critical processes affecting microplastic transport and to provide recommendations on where, when, and what to sample in rivers and transitional zones. We highlight priority locations such as salinity gradients, biologically active zones, and hydrodynamically diverse areas. Temporal guidance includes the duration of hydrodynamic and biological processes, study objectives (transport vs. retention), and sudden environmental disturbances such as floods or algal bloom collapses. For particle characterization, we evaluate shape descriptors and recommend recording at least the three principal dimensions, as they can be translated into quantitative shape descriptors relevant for modelling. Finally, we present a practical checklist outlining essential measurements for microplastics, water, sediment, additional substances, and surrounding conditions. Incorporating these insights into future monitoring campaigns will improve the ecological relevance and interpretability of microplastic monitoring.</t>
+  </si>
+  <si>
+    <t>Guidance and checklist</t>
+  </si>
+  <si>
+    <t>Comprehensive review up to August 2024 with harmonized recommendations on where, when, and what to sample in rivers and transitional zones.</t>
   </si>
 </sst>
 </file>
@@ -5108,7 +5129,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -5380,38 +5401,17 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="8" fillId="10" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="5" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -5434,19 +5434,30 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="6" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="8" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -5454,9 +5465,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="52">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -5908,6 +5916,9 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -5967,66 +5978,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}" name="Table2" displayName="Table2" ref="A2:BB188" totalsRowShown="0" headerRowBorderDxfId="51">
-  <autoFilter ref="A2:BB188" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}" name="Table2" displayName="Table2" ref="A2:BB189" totalsRowShown="0" headerRowBorderDxfId="51">
+  <autoFilter ref="A2:BB189" xr:uid="{D7F74609-08FF-44E4-8D38-7B6CD8B94E02}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:BB176">
     <sortCondition ref="A2:A176"/>
   </sortState>
   <tableColumns count="54">
     <tableColumn id="1" xr3:uid="{157273E0-51BF-4198-AAA3-2216EFF6F18E}" name="#" dataDxfId="50"/>
     <tableColumn id="2" xr3:uid="{A8B1C8EE-F997-46EF-A198-05152546D1B5}" name="Short Citation" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{07F5FB6A-A650-41C8-A3B3-26567DEDC704}" name="Year" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{0831BE7B-82A3-4CA6-9FE4-C5DE13BF7499}" name="Full Title" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{8BDF9B71-F522-49EF-94E8-E0F244981500}" name="DOI/URL" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{19E5A9BF-1647-47BE-84D8-E72FF78D4F00}" name="Primary Domain" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{1365C634-3EE3-40D0-812F-4BA4FAED29E5}" name="Primary Focus" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{338122AB-5BD8-4866-A37E-3D39FA6670A2}" name="Document Type" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{27C9A60F-C709-4EA8-89A1-9E39AE07E9C1}" name="Priority_x000a_Tier" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{1D524DA9-0888-49F2-8229-DF236A082D36}" name="Instrumentation Tags" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{5C25CF41-F23E-4963-91C6-24C3E65B7436}" name="Matrix Tags" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{07F5FB6A-A650-41C8-A3B3-26567DEDC704}" name="Year" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{0831BE7B-82A3-4CA6-9FE4-C5DE13BF7499}" name="Full Title" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{8BDF9B71-F522-49EF-94E8-E0F244981500}" name="DOI/URL" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{19E5A9BF-1647-47BE-84D8-E72FF78D4F00}" name="Primary Domain" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{1365C634-3EE3-40D0-812F-4BA4FAED29E5}" name="Primary Focus" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{338122AB-5BD8-4866-A37E-3D39FA6670A2}" name="Document Type" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{27C9A60F-C709-4EA8-89A1-9E39AE07E9C1}" name="Priority_x000a_Tier" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{1D524DA9-0888-49F2-8229-DF236A082D36}" name="Instrumentation Tags" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{5C25CF41-F23E-4963-91C6-24C3E65B7436}" name="Matrix Tags" dataDxfId="40"/>
     <tableColumn id="12" xr3:uid="{FF901B25-2718-4138-805C-8F6455E23A05}" name="Particle/Polymer Type Tags"/>
-    <tableColumn id="13" xr3:uid="{CEDE63B6-1DE0-4F1C-819A-19776FC8DC6E}" name="Target Receptor(s)" dataDxfId="40"/>
-    <tableColumn id="14" xr3:uid="{9A4E571D-A1F6-40DC-B704-E1294F7DAB36}" name="Definitions &amp;_x000a_Terminology" dataDxfId="39"/>
-    <tableColumn id="15" xr3:uid="{941447EA-878B-4190-B298-856AC8347372}" name="Problem Formulation_x000a_/ Framework" dataDxfId="38"/>
-    <tableColumn id="16" xr3:uid="{CB178553-686B-4C5E-97E2-8A02E5FD0D55}" name="Sampling_x000a_(Field Methods)" dataDxfId="37"/>
-    <tableColumn id="17" xr3:uid="{228CC6E5-F85A-43D4-9C0D-E113F9ACA161}" name="Matrix:_x000a_Drinking Water" dataDxfId="36"/>
-    <tableColumn id="18" xr3:uid="{B123E62B-3AC0-435F-9145-4C8127CAA77C}" name="Matrix: Surface Water" dataDxfId="35"/>
-    <tableColumn id="19" xr3:uid="{CEF38C2B-2F06-4E78-A092-E2FEB97C9F52}" name="Matrix: Surface Water - Lacustrine" dataDxfId="34"/>
-    <tableColumn id="20" xr3:uid="{3694A582-64F6-4477-A9D8-06177956C242}" name="Matrix: Surface Water - Riverine" dataDxfId="33"/>
-    <tableColumn id="21" xr3:uid="{F583F8B6-3B8E-4B25-A98F-419E5647A5EA}" name="Matrix: Surface Water - Marine" dataDxfId="32"/>
-    <tableColumn id="22" xr3:uid="{85C0E723-D5C6-4324-94BB-D0F3DCA9B995}" name="Matrix:_x000a_Wastewater" dataDxfId="31"/>
-    <tableColumn id="23" xr3:uid="{8220585C-5CF1-41AF-919C-4C99A59721F7}" name="Matrix: Groundwater" dataDxfId="30"/>
-    <tableColumn id="24" xr3:uid="{FEBA89A1-F5D0-4F0D-B25F-6FB85D7243C0}" name="Matrix: Biosolids" dataDxfId="29"/>
-    <tableColumn id="25" xr3:uid="{09AB8842-0DF4-4F69-9168-1E1EDBACD5ED}" name="Matrix:_x000a_Sediment" dataDxfId="28"/>
-    <tableColumn id="26" xr3:uid="{0B7FDDE7-15ED-49F7-85D5-EC288FFD9ABF}" name="Matrix:_x000a_Soil" dataDxfId="27"/>
-    <tableColumn id="27" xr3:uid="{5C63260E-F930-45B8-BBDD-70838E6E43F5}" name="Matrix:_x000a_Biota/Tissue" dataDxfId="26"/>
-    <tableColumn id="28" xr3:uid="{DCD27DA6-354F-4360-8C09-BD78208BA02A}" name="Matrix:_x000a_Air/Atmos." dataDxfId="25"/>
-    <tableColumn id="29" xr3:uid="{4184C4AC-BEC3-404E-ACC5-AED032740DFF}" name="Matrix:_x000a_Food/Dietary" dataDxfId="24"/>
-    <tableColumn id="30" xr3:uid="{0E8CD545-AFE9-4376-8F44-48E6F9FC2936}" name="Matrix:_x000a_Human Tissue/_x000a_Biomonitor" dataDxfId="23"/>
-    <tableColumn id="31" xr3:uid="{4FAB3A2F-40D5-4FA8-BFC4-CB409107DB63}" name="Sample Processing_x000a_/ Extraction" dataDxfId="22"/>
-    <tableColumn id="32" xr3:uid="{5E7A3CB2-36D4-4594-BFB7-9F49BAA3A2D2}" name="Sub-sampling" dataDxfId="21"/>
-    <tableColumn id="33" xr3:uid="{1555478C-CD74-4F0E-9374-B5B012702DD9}" name="Analytical_x000a_Methods (General)" dataDxfId="20"/>
-    <tableColumn id="34" xr3:uid="{5E9715CD-9A76-4D03-9048-0AF3B32A2499}" name="FTIR / IR_x000a_Spectroscopy" dataDxfId="19"/>
-    <tableColumn id="35" xr3:uid="{6EF7B799-0FBF-4A00-9379-8FEADFA4E38A}" name="Raman_x000a_Spectroscopy" dataDxfId="18"/>
-    <tableColumn id="36" xr3:uid="{9C42805B-BA1D-45C3-9788-C9FB01D3D549}" name="Py-GC-MS" dataDxfId="17"/>
-    <tableColumn id="37" xr3:uid="{8DA2DD01-42A0-4C44-AB7F-B4754280832F}" name="Imaging" dataDxfId="16"/>
-    <tableColumn id="38" xr3:uid="{BB38F2B1-716D-48CA-A962-EA86DA3F849A}" name="Material Standards - materials" dataDxfId="15"/>
-    <tableColumn id="53" xr3:uid="{2E043EA4-F707-4069-9455-F0555C524C97}" name="Material Standards - protocol" dataDxfId="14"/>
-    <tableColumn id="39" xr3:uid="{9D69D833-46AC-4D69-A3FE-62512232C633}" name="Blanks &amp;_x000a_Contamination_x000a_Control" dataDxfId="13"/>
-    <tableColumn id="40" xr3:uid="{9628E9F5-3972-4FE0-9F02-83F8F9AB87B8}" name="Data Analysis_x000a_&amp; Statistics" dataDxfId="12"/>
-    <tableColumn id="41" xr3:uid="{E08A5C14-9082-4603-A2E5-0F190EA86465}" name="Reporting &amp;_x000a_Harmonization" dataDxfId="11"/>
-    <tableColumn id="42" xr3:uid="{15B782A9-BA11-42A8-8714-5859A51B9793}" name="Databases &amp;_x000a_Data Sharing" dataDxfId="10"/>
-    <tableColumn id="43" xr3:uid="{38DF8C33-36D2-431F-BB1C-E55F8D19DC14}" name="Toxicology:_x000a_Study Design &amp;_x000a_Dosimetry" dataDxfId="9"/>
-    <tableColumn id="44" xr3:uid="{D753897E-2232-42BB-B6A0-E9664869043F}" name="Toxicology:_x000a_Effects Testing_x000a_Methods" dataDxfId="8"/>
-    <tableColumn id="55" xr3:uid="{E25D3005-678F-4519-BBBF-F84B844C6386}" name="Toxicology: Reporting &amp; Harmonization" dataDxfId="7"/>
-    <tableColumn id="54" xr3:uid="{794AF906-9949-4D89-A079-01CE5E48D018}" name="Toxicology: Databases &amp; Data Sharing" dataDxfId="6"/>
-    <tableColumn id="46" xr3:uid="{3158ED12-9442-4B00-8CEC-E9D37D8F4E2D}" name="Risk_x000a_Assessment /_x000a_Risk Char." dataDxfId="5"/>
-    <tableColumn id="47" xr3:uid="{0FD00342-A9D9-478F-9383-D2F6B853A44D}" name="Key Notes" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{CEDE63B6-1DE0-4F1C-819A-19776FC8DC6E}" name="Target Receptor(s)" dataDxfId="39"/>
+    <tableColumn id="14" xr3:uid="{9A4E571D-A1F6-40DC-B704-E1294F7DAB36}" name="Definitions &amp;_x000a_Terminology" dataDxfId="38"/>
+    <tableColumn id="15" xr3:uid="{941447EA-878B-4190-B298-856AC8347372}" name="Problem Formulation_x000a_/ Framework" dataDxfId="37"/>
+    <tableColumn id="16" xr3:uid="{CB178553-686B-4C5E-97E2-8A02E5FD0D55}" name="Sampling_x000a_(Field Methods)" dataDxfId="36"/>
+    <tableColumn id="17" xr3:uid="{228CC6E5-F85A-43D4-9C0D-E113F9ACA161}" name="Matrix:_x000a_Drinking Water" dataDxfId="35"/>
+    <tableColumn id="18" xr3:uid="{B123E62B-3AC0-435F-9145-4C8127CAA77C}" name="Matrix: Surface Water" dataDxfId="34"/>
+    <tableColumn id="19" xr3:uid="{CEF38C2B-2F06-4E78-A092-E2FEB97C9F52}" name="Matrix: Surface Water - Lacustrine" dataDxfId="33"/>
+    <tableColumn id="20" xr3:uid="{3694A582-64F6-4477-A9D8-06177956C242}" name="Matrix: Surface Water - Riverine" dataDxfId="32"/>
+    <tableColumn id="21" xr3:uid="{F583F8B6-3B8E-4B25-A98F-419E5647A5EA}" name="Matrix: Surface Water - Marine" dataDxfId="31"/>
+    <tableColumn id="22" xr3:uid="{85C0E723-D5C6-4324-94BB-D0F3DCA9B995}" name="Matrix:_x000a_Wastewater" dataDxfId="30"/>
+    <tableColumn id="23" xr3:uid="{8220585C-5CF1-41AF-919C-4C99A59721F7}" name="Matrix: Groundwater" dataDxfId="29"/>
+    <tableColumn id="24" xr3:uid="{FEBA89A1-F5D0-4F0D-B25F-6FB85D7243C0}" name="Matrix: Biosolids" dataDxfId="28"/>
+    <tableColumn id="25" xr3:uid="{09AB8842-0DF4-4F69-9168-1E1EDBACD5ED}" name="Matrix:_x000a_Sediment" dataDxfId="27"/>
+    <tableColumn id="26" xr3:uid="{0B7FDDE7-15ED-49F7-85D5-EC288FFD9ABF}" name="Matrix:_x000a_Soil" dataDxfId="26"/>
+    <tableColumn id="27" xr3:uid="{5C63260E-F930-45B8-BBDD-70838E6E43F5}" name="Matrix:_x000a_Biota/Tissue" dataDxfId="25"/>
+    <tableColumn id="28" xr3:uid="{DCD27DA6-354F-4360-8C09-BD78208BA02A}" name="Matrix:_x000a_Air/Atmos." dataDxfId="24"/>
+    <tableColumn id="29" xr3:uid="{4184C4AC-BEC3-404E-ACC5-AED032740DFF}" name="Matrix:_x000a_Food/Dietary" dataDxfId="23"/>
+    <tableColumn id="30" xr3:uid="{0E8CD545-AFE9-4376-8F44-48E6F9FC2936}" name="Matrix:_x000a_Human Tissue/_x000a_Biomonitor" dataDxfId="22"/>
+    <tableColumn id="31" xr3:uid="{4FAB3A2F-40D5-4FA8-BFC4-CB409107DB63}" name="Sample Processing_x000a_/ Extraction" dataDxfId="21"/>
+    <tableColumn id="32" xr3:uid="{5E7A3CB2-36D4-4594-BFB7-9F49BAA3A2D2}" name="Sub-sampling" dataDxfId="20"/>
+    <tableColumn id="33" xr3:uid="{1555478C-CD74-4F0E-9374-B5B012702DD9}" name="Analytical_x000a_Methods (General)" dataDxfId="19"/>
+    <tableColumn id="34" xr3:uid="{5E9715CD-9A76-4D03-9048-0AF3B32A2499}" name="FTIR / IR_x000a_Spectroscopy" dataDxfId="18"/>
+    <tableColumn id="35" xr3:uid="{6EF7B799-0FBF-4A00-9379-8FEADFA4E38A}" name="Raman_x000a_Spectroscopy" dataDxfId="17"/>
+    <tableColumn id="36" xr3:uid="{9C42805B-BA1D-45C3-9788-C9FB01D3D549}" name="Py-GC-MS" dataDxfId="16"/>
+    <tableColumn id="37" xr3:uid="{8DA2DD01-42A0-4C44-AB7F-B4754280832F}" name="Imaging" dataDxfId="15"/>
+    <tableColumn id="38" xr3:uid="{BB38F2B1-716D-48CA-A962-EA86DA3F849A}" name="Material Standards - materials" dataDxfId="14"/>
+    <tableColumn id="53" xr3:uid="{2E043EA4-F707-4069-9455-F0555C524C97}" name="Material Standards - protocol" dataDxfId="13"/>
+    <tableColumn id="39" xr3:uid="{9D69D833-46AC-4D69-A3FE-62512232C633}" name="Blanks &amp;_x000a_Contamination_x000a_Control" dataDxfId="12"/>
+    <tableColumn id="40" xr3:uid="{9628E9F5-3972-4FE0-9F02-83F8F9AB87B8}" name="Data Analysis_x000a_&amp; Statistics" dataDxfId="11"/>
+    <tableColumn id="41" xr3:uid="{E08A5C14-9082-4603-A2E5-0F190EA86465}" name="Reporting &amp;_x000a_Harmonization" dataDxfId="10"/>
+    <tableColumn id="42" xr3:uid="{15B782A9-BA11-42A8-8714-5859A51B9793}" name="Databases &amp;_x000a_Data Sharing" dataDxfId="9"/>
+    <tableColumn id="43" xr3:uid="{38DF8C33-36D2-431F-BB1C-E55F8D19DC14}" name="Toxicology:_x000a_Study Design &amp;_x000a_Dosimetry" dataDxfId="8"/>
+    <tableColumn id="44" xr3:uid="{D753897E-2232-42BB-B6A0-E9664869043F}" name="Toxicology:_x000a_Effects Testing_x000a_Methods" dataDxfId="7"/>
+    <tableColumn id="55" xr3:uid="{E25D3005-678F-4519-BBBF-F84B844C6386}" name="Toxicology: Reporting &amp; Harmonization" dataDxfId="6"/>
+    <tableColumn id="54" xr3:uid="{794AF906-9949-4D89-A079-01CE5E48D018}" name="Toxicology: Databases &amp; Data Sharing" dataDxfId="5"/>
+    <tableColumn id="46" xr3:uid="{3158ED12-9442-4B00-8CEC-E9D37D8F4E2D}" name="Risk_x000a_Assessment /_x000a_Risk Char." dataDxfId="4"/>
+    <tableColumn id="47" xr3:uid="{0FD00342-A9D9-478F-9383-D2F6B853A44D}" name="Key Notes" dataDxfId="3"/>
     <tableColumn id="48" xr3:uid="{4BE1F33B-7E0D-4F32-B492-F28D43B48E54}" name="Scope"/>
     <tableColumn id="49" xr3:uid="{D2279340-23C3-4EE5-8570-F5244F0755EE}" name="Status"/>
-    <tableColumn id="50" xr3:uid="{81909305-108A-4B91-BCE6-89E889DE39A8}" name="Particle_x000a_Size Range" dataDxfId="3"/>
-    <tableColumn id="51" xr3:uid="{2AECE94C-1735-4B86-999E-F6C4105FFCFE}" name="Key Metrics /_x000a_Output" dataDxfId="2"/>
-    <tableColumn id="52" xr3:uid="{2DD3D9F5-1988-478B-BB45-CD54211D41B5}" name="Abstract" dataDxfId="1"/>
+    <tableColumn id="50" xr3:uid="{81909305-108A-4B91-BCE6-89E889DE39A8}" name="Particle_x000a_Size Range" dataDxfId="2"/>
+    <tableColumn id="51" xr3:uid="{2AECE94C-1735-4B86-999E-F6C4105FFCFE}" name="Key Metrics /_x000a_Output" dataDxfId="1"/>
+    <tableColumn id="52" xr3:uid="{2DD3D9F5-1988-478B-BB45-CD54211D41B5}" name="Abstract" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6365,31 +6376,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:54" ht="66.599999999999994" hidden="1" customHeight="1">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="106" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="96"/>
+      <c r="B1" s="107"/>
       <c r="C1" s="97"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="98"/>
-      <c r="F1" s="99" t="s">
+      <c r="D1" s="107"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="109" t="s">
         <v>37</v>
       </c>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
-      <c r="I1" s="100"/>
-      <c r="J1" s="100"/>
-      <c r="K1" s="96"/>
-      <c r="L1" s="96"/>
-      <c r="M1" s="98"/>
-      <c r="N1" s="101" t="s">
+      <c r="G1" s="110"/>
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="107"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="111" t="s">
         <v>38</v>
       </c>
-      <c r="O1" s="102"/>
+      <c r="O1" s="98"/>
       <c r="P1" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="Q1" s="103" t="s">
+      <c r="Q1" s="112" t="s">
         <v>40</v>
       </c>
       <c r="R1" s="97"/>
@@ -6404,36 +6415,36 @@
       <c r="AA1" s="97"/>
       <c r="AB1" s="97"/>
       <c r="AC1" s="97"/>
-      <c r="AD1" s="102"/>
-      <c r="AE1" s="104" t="s">
+      <c r="AD1" s="98"/>
+      <c r="AE1" s="113" t="s">
         <v>41</v>
       </c>
-      <c r="AF1" s="102"/>
-      <c r="AG1" s="105" t="s">
+      <c r="AF1" s="98"/>
+      <c r="AG1" s="96" t="s">
         <v>42</v>
       </c>
       <c r="AH1" s="97"/>
       <c r="AI1" s="97"/>
-      <c r="AJ1" s="102"/>
+      <c r="AJ1" s="98"/>
       <c r="AK1" s="15"/>
       <c r="AL1" s="16" t="s">
         <v>43</v>
       </c>
       <c r="AM1" s="78"/>
-      <c r="AN1" s="106" t="s">
+      <c r="AN1" s="99" t="s">
         <v>44</v>
       </c>
-      <c r="AO1" s="102"/>
-      <c r="AP1" s="107" t="s">
+      <c r="AO1" s="98"/>
+      <c r="AP1" s="100" t="s">
         <v>45</v>
       </c>
-      <c r="AQ1" s="102"/>
-      <c r="AR1" s="108" t="s">
+      <c r="AQ1" s="98"/>
+      <c r="AR1" s="101" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" s="109"/>
-      <c r="AT1" s="109"/>
-      <c r="AU1" s="109"/>
+      <c r="AS1" s="102"/>
+      <c r="AT1" s="102"/>
+      <c r="AU1" s="102"/>
       <c r="AV1" s="17" t="s">
         <v>44</v>
       </c>
@@ -6442,11 +6453,11 @@
       </c>
       <c r="AX1" s="19"/>
       <c r="AY1" s="19"/>
-      <c r="AZ1" s="110" t="s">
+      <c r="AZ1" s="103" t="s">
         <v>48</v>
       </c>
-      <c r="BA1" s="111"/>
-      <c r="BB1" s="112"/>
+      <c r="BA1" s="104"/>
+      <c r="BB1" s="105"/>
     </row>
     <row r="2" spans="1:54" s="4" customFormat="1" ht="57.75" customHeight="1">
       <c r="A2" s="20" t="s">
@@ -6619,7 +6630,7 @@
       <c r="B3" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="113">
+      <c r="C3" s="37">
         <v>2009</v>
       </c>
       <c r="D3" s="37" t="s">
@@ -6717,7 +6728,7 @@
       <c r="B4" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="113">
+      <c r="C4" s="37">
         <v>2013</v>
       </c>
       <c r="D4" s="37" t="s">
@@ -6825,7 +6836,7 @@
       <c r="B5" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="113">
+      <c r="C5" s="37">
         <v>2015</v>
       </c>
       <c r="D5" s="37" t="s">
@@ -6929,7 +6940,7 @@
       <c r="B6" s="37" t="s">
         <v>133</v>
       </c>
-      <c r="C6" s="113">
+      <c r="C6" s="37">
         <v>2023</v>
       </c>
       <c r="D6" s="37" t="s">
@@ -7031,7 +7042,7 @@
       <c r="B7" s="37" t="s">
         <v>141</v>
       </c>
-      <c r="C7" s="113">
+      <c r="C7" s="37">
         <v>2025</v>
       </c>
       <c r="D7" s="37" t="s">
@@ -7135,7 +7146,7 @@
       <c r="B8" s="37" t="s">
         <v>150</v>
       </c>
-      <c r="C8" s="113">
+      <c r="C8" s="37">
         <v>2024</v>
       </c>
       <c r="D8" s="37" t="s">
@@ -7241,7 +7252,7 @@
       <c r="B9" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="C9" s="113">
+      <c r="C9" s="37">
         <v>2023</v>
       </c>
       <c r="D9" s="37" t="s">
@@ -7347,7 +7358,7 @@
       <c r="B10" s="37" t="s">
         <v>163</v>
       </c>
-      <c r="C10" s="113">
+      <c r="C10" s="37">
         <v>2021</v>
       </c>
       <c r="D10" s="37" t="s">
@@ -7441,7 +7452,7 @@
       <c r="B11" s="37" t="s">
         <v>173</v>
       </c>
-      <c r="C11" s="113">
+      <c r="C11" s="37">
         <v>2025</v>
       </c>
       <c r="D11" s="37" t="s">
@@ -7537,7 +7548,7 @@
       <c r="B12" s="37" t="s">
         <v>180</v>
       </c>
-      <c r="C12" s="113">
+      <c r="C12" s="37">
         <v>2022</v>
       </c>
       <c r="D12" s="37" t="s">
@@ -7633,7 +7644,7 @@
       <c r="B13" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="C13" s="113">
+      <c r="C13" s="37">
         <v>2025</v>
       </c>
       <c r="D13" s="37" t="s">
@@ -7729,7 +7740,7 @@
       <c r="B14" s="37" t="s">
         <v>196</v>
       </c>
-      <c r="C14" s="113">
+      <c r="C14" s="37">
         <v>2025</v>
       </c>
       <c r="D14" s="37" t="s">
@@ -7821,7 +7832,7 @@
       <c r="B15" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="C15" s="113">
+      <c r="C15" s="37">
         <v>2020</v>
       </c>
       <c r="D15" s="37" t="s">
@@ -7915,7 +7926,7 @@
       <c r="B16" s="37" t="s">
         <v>212</v>
       </c>
-      <c r="C16" s="113">
+      <c r="C16" s="37">
         <v>2011</v>
       </c>
       <c r="D16" s="37" t="s">
@@ -8003,7 +8014,7 @@
       <c r="B17" s="37" t="s">
         <v>218</v>
       </c>
-      <c r="C17" s="113">
+      <c r="C17" s="37">
         <v>2019</v>
       </c>
       <c r="D17" s="37" t="s">
@@ -8095,7 +8106,7 @@
       <c r="B18" s="37" t="s">
         <v>226</v>
       </c>
-      <c r="C18" s="113">
+      <c r="C18" s="37">
         <v>2017</v>
       </c>
       <c r="D18" s="37" t="s">
@@ -8195,7 +8206,7 @@
       <c r="B19" s="37" t="s">
         <v>237</v>
       </c>
-      <c r="C19" s="113">
+      <c r="C19" s="37">
         <v>2022</v>
       </c>
       <c r="D19" s="37" t="s">
@@ -8287,7 +8298,7 @@
       <c r="B20" s="37" t="s">
         <v>245</v>
       </c>
-      <c r="C20" s="113">
+      <c r="C20" s="37">
         <v>2023</v>
       </c>
       <c r="D20" s="37" t="s">
@@ -8383,7 +8394,7 @@
       <c r="B21" s="37" t="s">
         <v>251</v>
       </c>
-      <c r="C21" s="113">
+      <c r="C21" s="37">
         <v>2024</v>
       </c>
       <c r="D21" s="37" t="s">
@@ -8477,7 +8488,7 @@
       <c r="B22" s="37" t="s">
         <v>256</v>
       </c>
-      <c r="C22" s="113">
+      <c r="C22" s="37">
         <v>2024</v>
       </c>
       <c r="D22" s="37" t="s">
@@ -8563,7 +8574,7 @@
       <c r="B23" s="37" t="s">
         <v>261</v>
       </c>
-      <c r="C23" s="113">
+      <c r="C23" s="37">
         <v>2019</v>
       </c>
       <c r="D23" s="37" t="s">
@@ -8661,7 +8672,7 @@
       <c r="B24" s="37" t="s">
         <v>267</v>
       </c>
-      <c r="C24" s="113">
+      <c r="C24" s="37">
         <v>2022</v>
       </c>
       <c r="D24" s="37" t="s">
@@ -8755,7 +8766,7 @@
       <c r="B25" s="37" t="s">
         <v>275</v>
       </c>
-      <c r="C25" s="113">
+      <c r="C25" s="37">
         <v>2025</v>
       </c>
       <c r="D25" s="37" t="s">
@@ -8845,7 +8856,7 @@
       <c r="B26" s="37" t="s">
         <v>283</v>
       </c>
-      <c r="C26" s="113">
+      <c r="C26" s="37">
         <v>2021</v>
       </c>
       <c r="D26" s="37" t="s">
@@ -8941,7 +8952,7 @@
       <c r="B27" s="37" t="s">
         <v>290</v>
       </c>
-      <c r="C27" s="113">
+      <c r="C27" s="37">
         <v>2024</v>
       </c>
       <c r="D27" s="37" t="s">
@@ -9031,7 +9042,7 @@
       <c r="B28" s="37" t="s">
         <v>299</v>
       </c>
-      <c r="C28" s="113">
+      <c r="C28" s="37">
         <v>2020</v>
       </c>
       <c r="D28" s="37" t="s">
@@ -9127,7 +9138,7 @@
       <c r="B29" s="37" t="s">
         <v>305</v>
       </c>
-      <c r="C29" s="113">
+      <c r="C29" s="37">
         <v>2025</v>
       </c>
       <c r="D29" s="37" t="s">
@@ -9225,7 +9236,7 @@
       <c r="B30" s="37" t="s">
         <v>312</v>
       </c>
-      <c r="C30" s="113">
+      <c r="C30" s="37">
         <v>2025</v>
       </c>
       <c r="D30" s="37" t="s">
@@ -9325,7 +9336,7 @@
       <c r="B31" s="37" t="s">
         <v>1350</v>
       </c>
-      <c r="C31" s="113">
+      <c r="C31" s="37">
         <v>2022</v>
       </c>
       <c r="D31" s="37" t="s">
@@ -9425,7 +9436,7 @@
       <c r="B32" s="37" t="s">
         <v>326</v>
       </c>
-      <c r="C32" s="113">
+      <c r="C32" s="37">
         <v>2024</v>
       </c>
       <c r="D32" s="37" t="s">
@@ -9515,7 +9526,7 @@
       <c r="B33" s="37" t="s">
         <v>333</v>
       </c>
-      <c r="C33" s="113">
+      <c r="C33" s="37">
         <v>2020</v>
       </c>
       <c r="D33" s="37" t="s">
@@ -9635,7 +9646,7 @@
       <c r="B34" s="37" t="s">
         <v>341</v>
       </c>
-      <c r="C34" s="113">
+      <c r="C34" s="37">
         <v>2020</v>
       </c>
       <c r="D34" s="37" t="s">
@@ -9753,7 +9764,7 @@
       <c r="B35" s="37" t="s">
         <v>348</v>
       </c>
-      <c r="C35" s="113">
+      <c r="C35" s="37">
         <v>2023</v>
       </c>
       <c r="D35" s="37" t="s">
@@ -9847,7 +9858,7 @@
       <c r="B36" s="37" t="s">
         <v>354</v>
       </c>
-      <c r="C36" s="113">
+      <c r="C36" s="37">
         <v>2024</v>
       </c>
       <c r="D36" s="37" t="s">
@@ -9939,7 +9950,7 @@
       <c r="B37" s="37" t="s">
         <v>362</v>
       </c>
-      <c r="C37" s="113">
+      <c r="C37" s="37">
         <v>2019</v>
       </c>
       <c r="D37" s="37" t="s">
@@ -10047,7 +10058,7 @@
       <c r="B38" s="37" t="s">
         <v>369</v>
       </c>
-      <c r="C38" s="113">
+      <c r="C38" s="37">
         <v>2019</v>
       </c>
       <c r="D38" s="37" t="s">
@@ -10145,7 +10156,7 @@
       <c r="B39" s="37" t="s">
         <v>377</v>
       </c>
-      <c r="C39" s="113">
+      <c r="C39" s="37">
         <v>2026</v>
       </c>
       <c r="D39" s="37" t="s">
@@ -10243,7 +10254,7 @@
       <c r="B40" s="37" t="s">
         <v>385</v>
       </c>
-      <c r="C40" s="113">
+      <c r="C40" s="37">
         <v>2021</v>
       </c>
       <c r="D40" s="37" t="s">
@@ -10339,7 +10350,7 @@
       <c r="B41" s="37" t="s">
         <v>393</v>
       </c>
-      <c r="C41" s="113">
+      <c r="C41" s="37">
         <v>2020</v>
       </c>
       <c r="D41" s="37" t="s">
@@ -10439,7 +10450,7 @@
       <c r="B42" s="37" t="s">
         <v>399</v>
       </c>
-      <c r="C42" s="113">
+      <c r="C42" s="37">
         <v>2026</v>
       </c>
       <c r="D42" s="37" t="s">
@@ -10531,7 +10542,7 @@
       <c r="B43" s="37" t="s">
         <v>406</v>
       </c>
-      <c r="C43" s="113">
+      <c r="C43" s="37">
         <v>2022</v>
       </c>
       <c r="D43" s="37" t="s">
@@ -10629,7 +10640,7 @@
       <c r="B44" s="37" t="s">
         <v>413</v>
       </c>
-      <c r="C44" s="113">
+      <c r="C44" s="37">
         <v>2021</v>
       </c>
       <c r="D44" s="37" t="s">
@@ -10723,7 +10734,7 @@
       <c r="B45" s="37" t="s">
         <v>420</v>
       </c>
-      <c r="C45" s="113">
+      <c r="C45" s="37">
         <v>2022</v>
       </c>
       <c r="D45" s="37" t="s">
@@ -10815,7 +10826,7 @@
       <c r="B46" s="37" t="s">
         <v>377</v>
       </c>
-      <c r="C46" s="113">
+      <c r="C46" s="37">
         <v>2026</v>
       </c>
       <c r="D46" s="37" t="s">
@@ -10909,7 +10920,7 @@
       <c r="B47" s="37" t="s">
         <v>432</v>
       </c>
-      <c r="C47" s="113">
+      <c r="C47" s="37">
         <v>2022</v>
       </c>
       <c r="D47" s="37" t="s">
@@ -11001,7 +11012,7 @@
       <c r="B48" s="37" t="s">
         <v>439</v>
       </c>
-      <c r="C48" s="113">
+      <c r="C48" s="37">
         <v>2025</v>
       </c>
       <c r="D48" s="37" t="s">
@@ -11105,7 +11116,7 @@
       <c r="B49" s="37" t="s">
         <v>449</v>
       </c>
-      <c r="C49" s="113">
+      <c r="C49" s="37">
         <v>2022</v>
       </c>
       <c r="D49" s="37" t="s">
@@ -11199,7 +11210,7 @@
       <c r="B50" s="37" t="s">
         <v>456</v>
       </c>
-      <c r="C50" s="113">
+      <c r="C50" s="37">
         <v>2019</v>
       </c>
       <c r="D50" s="37" t="s">
@@ -11293,7 +11304,7 @@
       <c r="B51" s="37" t="s">
         <v>464</v>
       </c>
-      <c r="C51" s="113">
+      <c r="C51" s="37">
         <v>2023</v>
       </c>
       <c r="D51" s="37" t="s">
@@ -11387,7 +11398,7 @@
       <c r="B52" s="37" t="s">
         <v>473</v>
       </c>
-      <c r="C52" s="113">
+      <c r="C52" s="37">
         <v>2021</v>
       </c>
       <c r="D52" s="37" t="s">
@@ -11483,7 +11494,7 @@
       <c r="B53" s="37" t="s">
         <v>479</v>
       </c>
-      <c r="C53" s="113">
+      <c r="C53" s="37">
         <v>2023</v>
       </c>
       <c r="D53" s="37" t="s">
@@ -11593,7 +11604,7 @@
       <c r="B54" s="37" t="s">
         <v>486</v>
       </c>
-      <c r="C54" s="113">
+      <c r="C54" s="37">
         <v>2021</v>
       </c>
       <c r="D54" s="37" t="s">
@@ -11685,7 +11696,7 @@
       <c r="B55" s="37" t="s">
         <v>494</v>
       </c>
-      <c r="C55" s="113">
+      <c r="C55" s="37">
         <v>2021</v>
       </c>
       <c r="D55" s="37" t="s">
@@ -11779,7 +11790,7 @@
       <c r="B56" s="37" t="s">
         <v>501</v>
       </c>
-      <c r="C56" s="113">
+      <c r="C56" s="37">
         <v>2019</v>
       </c>
       <c r="D56" s="37" t="s">
@@ -11883,7 +11894,7 @@
       <c r="B57" s="37" t="s">
         <v>508</v>
       </c>
-      <c r="C57" s="113">
+      <c r="C57" s="37">
         <v>2015</v>
       </c>
       <c r="D57" s="37" t="s">
@@ -11979,7 +11990,7 @@
       <c r="B58" s="37" t="s">
         <v>514</v>
       </c>
-      <c r="C58" s="113">
+      <c r="C58" s="37">
         <v>2016</v>
       </c>
       <c r="D58" s="37" t="s">
@@ -12079,7 +12090,7 @@
       <c r="B59" s="37" t="s">
         <v>520</v>
       </c>
-      <c r="C59" s="113">
+      <c r="C59" s="37">
         <v>2019</v>
       </c>
       <c r="D59" s="37" t="s">
@@ -12169,7 +12180,7 @@
       <c r="B60" s="37" t="s">
         <v>525</v>
       </c>
-      <c r="C60" s="113">
+      <c r="C60" s="37">
         <v>2022</v>
       </c>
       <c r="D60" s="37" t="s">
@@ -12265,7 +12276,7 @@
       <c r="B61" s="37" t="s">
         <v>532</v>
       </c>
-      <c r="C61" s="113">
+      <c r="C61" s="37">
         <v>2015</v>
       </c>
       <c r="D61" s="37" t="s">
@@ -12359,7 +12370,7 @@
       <c r="B62" s="37" t="s">
         <v>540</v>
       </c>
-      <c r="C62" s="113">
+      <c r="C62" s="37">
         <v>2024</v>
       </c>
       <c r="D62" s="37" t="s">
@@ -12451,7 +12462,7 @@
       <c r="B63" s="37" t="s">
         <v>547</v>
       </c>
-      <c r="C63" s="113">
+      <c r="C63" s="37">
         <v>2021</v>
       </c>
       <c r="D63" s="37" t="s">
@@ -12545,7 +12556,7 @@
       <c r="B64" s="37" t="s">
         <v>554</v>
       </c>
-      <c r="C64" s="113">
+      <c r="C64" s="37">
         <v>2023</v>
       </c>
       <c r="D64" s="37" t="s">
@@ -12651,7 +12662,7 @@
       <c r="B65" s="37" t="s">
         <v>562</v>
       </c>
-      <c r="C65" s="113">
+      <c r="C65" s="37">
         <v>2020</v>
       </c>
       <c r="D65" s="37" t="s">
@@ -12747,7 +12758,7 @@
       <c r="B66" s="37" t="s">
         <v>569</v>
       </c>
-      <c r="C66" s="113">
+      <c r="C66" s="37">
         <v>2024</v>
       </c>
       <c r="D66" s="37" t="s">
@@ -12853,7 +12864,7 @@
       <c r="B67" s="37" t="s">
         <v>577</v>
       </c>
-      <c r="C67" s="113">
+      <c r="C67" s="37">
         <v>2023</v>
       </c>
       <c r="D67" s="37" t="s">
@@ -12961,7 +12972,7 @@
       <c r="B68" s="37" t="s">
         <v>583</v>
       </c>
-      <c r="C68" s="113">
+      <c r="C68" s="37">
         <v>2025</v>
       </c>
       <c r="D68" s="37" t="s">
@@ -13073,7 +13084,7 @@
       <c r="B69" s="37" t="s">
         <v>590</v>
       </c>
-      <c r="C69" s="113">
+      <c r="C69" s="37">
         <v>2026</v>
       </c>
       <c r="D69" s="37" t="s">
@@ -13171,7 +13182,7 @@
       <c r="B70" s="37" t="s">
         <v>597</v>
       </c>
-      <c r="C70" s="113">
+      <c r="C70" s="37">
         <v>2023</v>
       </c>
       <c r="D70" s="37" t="s">
@@ -13261,7 +13272,7 @@
       <c r="B71" s="58" t="s">
         <v>605</v>
       </c>
-      <c r="C71" s="114">
+      <c r="C71" s="95">
         <v>2026</v>
       </c>
       <c r="D71" s="58" t="s">
@@ -13351,7 +13362,7 @@
       <c r="B72" s="37" t="s">
         <v>613</v>
       </c>
-      <c r="C72" s="113">
+      <c r="C72" s="37">
         <v>2024</v>
       </c>
       <c r="D72" s="37" t="s">
@@ -13441,7 +13452,7 @@
       <c r="B73" s="37" t="s">
         <v>619</v>
       </c>
-      <c r="C73" s="113">
+      <c r="C73" s="37">
         <v>2024</v>
       </c>
       <c r="D73" s="37" t="s">
@@ -13533,7 +13544,7 @@
       <c r="B74" s="37" t="s">
         <v>627</v>
       </c>
-      <c r="C74" s="113">
+      <c r="C74" s="37">
         <v>2023</v>
       </c>
       <c r="D74" s="37" t="s">
@@ -13623,7 +13634,7 @@
       <c r="B75" s="37" t="s">
         <v>633</v>
       </c>
-      <c r="C75" s="113">
+      <c r="C75" s="37">
         <v>2017</v>
       </c>
       <c r="D75" s="37" t="s">
@@ -13719,7 +13730,7 @@
       <c r="B76" s="37" t="s">
         <v>641</v>
       </c>
-      <c r="C76" s="113">
+      <c r="C76" s="37">
         <v>2023</v>
       </c>
       <c r="D76" s="37" t="s">
@@ -13811,7 +13822,7 @@
       <c r="B77" s="37" t="s">
         <v>649</v>
       </c>
-      <c r="C77" s="113">
+      <c r="C77" s="37">
         <v>2023</v>
       </c>
       <c r="D77" s="37" t="s">
@@ -13905,7 +13916,7 @@
       <c r="B78" s="37" t="s">
         <v>656</v>
       </c>
-      <c r="C78" s="113">
+      <c r="C78" s="37">
         <v>2023</v>
       </c>
       <c r="D78" s="37" t="s">
@@ -13997,7 +14008,7 @@
       <c r="B79" s="37" t="s">
         <v>661</v>
       </c>
-      <c r="C79" s="113">
+      <c r="C79" s="37">
         <v>2025</v>
       </c>
       <c r="D79" s="37" t="s">
@@ -14099,7 +14110,7 @@
       <c r="B80" s="37" t="s">
         <v>666</v>
       </c>
-      <c r="C80" s="113">
+      <c r="C80" s="37">
         <v>2024</v>
       </c>
       <c r="D80" s="37" t="s">
@@ -14191,7 +14202,7 @@
       <c r="B81" s="37" t="s">
         <v>674</v>
       </c>
-      <c r="C81" s="113">
+      <c r="C81" s="37">
         <v>2019</v>
       </c>
       <c r="D81" s="37" t="s">
@@ -14283,7 +14294,7 @@
       <c r="B82" s="37" t="s">
         <v>682</v>
       </c>
-      <c r="C82" s="113">
+      <c r="C82" s="37">
         <v>2017</v>
       </c>
       <c r="D82" s="37" t="s">
@@ -14379,7 +14390,7 @@
       <c r="B83" s="58" t="s">
         <v>688</v>
       </c>
-      <c r="C83" s="114">
+      <c r="C83" s="95">
         <v>2026</v>
       </c>
       <c r="D83" s="58" t="s">
@@ -14469,7 +14480,7 @@
       <c r="B84" s="37" t="s">
         <v>694</v>
       </c>
-      <c r="C84" s="113">
+      <c r="C84" s="37">
         <v>2025</v>
       </c>
       <c r="D84" s="37" t="s">
@@ -14589,7 +14600,7 @@
       <c r="B85" s="37" t="s">
         <v>703</v>
       </c>
-      <c r="C85" s="113">
+      <c r="C85" s="37">
         <v>2023</v>
       </c>
       <c r="D85" s="37" t="s">
@@ -14679,7 +14690,7 @@
       <c r="B86" s="37" t="s">
         <v>709</v>
       </c>
-      <c r="C86" s="113">
+      <c r="C86" s="37">
         <v>2025</v>
       </c>
       <c r="D86" s="37" t="s">
@@ -14769,7 +14780,7 @@
       <c r="B87" s="37" t="s">
         <v>714</v>
       </c>
-      <c r="C87" s="113">
+      <c r="C87" s="37">
         <v>2024</v>
       </c>
       <c r="D87" s="37" t="s">
@@ -14863,7 +14874,7 @@
       <c r="B88" s="37" t="s">
         <v>722</v>
       </c>
-      <c r="C88" s="113">
+      <c r="C88" s="37">
         <v>2022</v>
       </c>
       <c r="D88" s="37" t="s">
@@ -14955,7 +14966,7 @@
       <c r="B89" s="37" t="s">
         <v>731</v>
       </c>
-      <c r="C89" s="113">
+      <c r="C89" s="37">
         <v>2019</v>
       </c>
       <c r="D89" s="37" t="s">
@@ -15055,7 +15066,7 @@
       <c r="B90" s="37" t="s">
         <v>739</v>
       </c>
-      <c r="C90" s="113">
+      <c r="C90" s="37">
         <v>2026</v>
       </c>
       <c r="D90" s="37" t="s">
@@ -15151,7 +15162,7 @@
       <c r="B91" s="58" t="s">
         <v>747</v>
       </c>
-      <c r="C91" s="114">
+      <c r="C91" s="95">
         <v>2026</v>
       </c>
       <c r="D91" s="61" t="s">
@@ -15245,7 +15256,7 @@
       <c r="B92" s="37" t="s">
         <v>753</v>
       </c>
-      <c r="C92" s="113">
+      <c r="C92" s="37">
         <v>2017</v>
       </c>
       <c r="D92" s="37" t="s">
@@ -15339,7 +15350,7 @@
       <c r="B93" s="37" t="s">
         <v>760</v>
       </c>
-      <c r="C93" s="113">
+      <c r="C93" s="37">
         <v>2022</v>
       </c>
       <c r="D93" s="37" t="s">
@@ -15439,7 +15450,7 @@
       <c r="B94" s="37" t="s">
         <v>767</v>
       </c>
-      <c r="C94" s="113">
+      <c r="C94" s="37">
         <v>2021</v>
       </c>
       <c r="D94" s="37" t="s">
@@ -15531,7 +15542,7 @@
       <c r="B95" s="37" t="s">
         <v>776</v>
       </c>
-      <c r="C95" s="113">
+      <c r="C95" s="37">
         <v>2023</v>
       </c>
       <c r="D95" s="37" t="s">
@@ -15619,7 +15630,7 @@
       <c r="B96" s="37" t="s">
         <v>783</v>
       </c>
-      <c r="C96" s="113">
+      <c r="C96" s="37">
         <v>2025</v>
       </c>
       <c r="D96" s="37" t="s">
@@ -15711,7 +15722,7 @@
       <c r="B97" s="37" t="s">
         <v>791</v>
       </c>
-      <c r="C97" s="113">
+      <c r="C97" s="37">
         <v>2025</v>
       </c>
       <c r="D97" s="37" t="s">
@@ -15811,7 +15822,7 @@
       <c r="B98" s="37" t="s">
         <v>799</v>
       </c>
-      <c r="C98" s="113">
+      <c r="C98" s="37">
         <v>2025</v>
       </c>
       <c r="D98" s="37" t="s">
@@ -15905,7 +15916,7 @@
       <c r="B99" s="37" t="s">
         <v>806</v>
       </c>
-      <c r="C99" s="113">
+      <c r="C99" s="37">
         <v>2020</v>
       </c>
       <c r="D99" s="37" t="s">
@@ -16003,7 +16014,7 @@
       <c r="B100" s="37" t="s">
         <v>814</v>
       </c>
-      <c r="C100" s="113">
+      <c r="C100" s="37">
         <v>2021</v>
       </c>
       <c r="D100" s="37" t="s">
@@ -16097,7 +16108,7 @@
       <c r="B101" s="37" t="s">
         <v>820</v>
       </c>
-      <c r="C101" s="113">
+      <c r="C101" s="37">
         <v>2022</v>
       </c>
       <c r="D101" s="37" t="s">
@@ -16193,7 +16204,7 @@
       <c r="B102" s="37" t="s">
         <v>827</v>
       </c>
-      <c r="C102" s="113">
+      <c r="C102" s="37">
         <v>2025</v>
       </c>
       <c r="D102" s="37" t="s">
@@ -16287,7 +16298,7 @@
       <c r="B103" s="37" t="s">
         <v>834</v>
       </c>
-      <c r="C103" s="113">
+      <c r="C103" s="37">
         <v>2025</v>
       </c>
       <c r="D103" s="37" t="s">
@@ -16385,7 +16396,7 @@
       <c r="B104" s="37" t="s">
         <v>841</v>
       </c>
-      <c r="C104" s="113">
+      <c r="C104" s="37">
         <v>2026</v>
       </c>
       <c r="D104" s="37" t="s">
@@ -16477,7 +16488,7 @@
       <c r="B105" s="37" t="s">
         <v>848</v>
       </c>
-      <c r="C105" s="113">
+      <c r="C105" s="37">
         <v>2021</v>
       </c>
       <c r="D105" s="37" t="s">
@@ -16567,7 +16578,7 @@
       <c r="B106" s="37" t="s">
         <v>856</v>
       </c>
-      <c r="C106" s="113">
+      <c r="C106" s="37">
         <v>2025</v>
       </c>
       <c r="D106" s="37" t="s">
@@ -16661,7 +16672,7 @@
       <c r="B107" s="37" t="s">
         <v>863</v>
       </c>
-      <c r="C107" s="113">
+      <c r="C107" s="37">
         <v>2022</v>
       </c>
       <c r="D107" s="37" t="s">
@@ -16755,7 +16766,7 @@
       <c r="B108" s="37" t="s">
         <v>870</v>
       </c>
-      <c r="C108" s="113">
+      <c r="C108" s="37">
         <v>2021</v>
       </c>
       <c r="D108" s="37" t="s">
@@ -16847,7 +16858,7 @@
       <c r="B109" s="37" t="s">
         <v>877</v>
       </c>
-      <c r="C109" s="113">
+      <c r="C109" s="37">
         <v>2021</v>
       </c>
       <c r="D109" s="37" t="s">
@@ -16955,7 +16966,7 @@
       <c r="B110" s="37" t="s">
         <v>884</v>
       </c>
-      <c r="C110" s="113">
+      <c r="C110" s="37">
         <v>2025</v>
       </c>
       <c r="D110" s="37" t="s">
@@ -17061,7 +17072,7 @@
       <c r="B111" s="37" t="s">
         <v>891</v>
       </c>
-      <c r="C111" s="113">
+      <c r="C111" s="37">
         <v>2022</v>
       </c>
       <c r="D111" s="37" t="s">
@@ -17157,7 +17168,7 @@
       <c r="B112" s="37" t="s">
         <v>898</v>
       </c>
-      <c r="C112" s="113">
+      <c r="C112" s="37">
         <v>2026</v>
       </c>
       <c r="D112" s="37" t="s">
@@ -17249,7 +17260,7 @@
       <c r="B113" s="37" t="s">
         <v>903</v>
       </c>
-      <c r="C113" s="113">
+      <c r="C113" s="37">
         <v>2022</v>
       </c>
       <c r="D113" s="37" t="s">
@@ -17351,7 +17362,7 @@
       <c r="B114" s="37" t="s">
         <v>912</v>
       </c>
-      <c r="C114" s="113">
+      <c r="C114" s="37">
         <v>2020</v>
       </c>
       <c r="D114" s="37" t="s">
@@ -17445,7 +17456,7 @@
       <c r="B115" s="37" t="s">
         <v>918</v>
       </c>
-      <c r="C115" s="113">
+      <c r="C115" s="37">
         <v>2019</v>
       </c>
       <c r="D115" s="37" t="s">
@@ -17535,7 +17546,7 @@
       <c r="B116" s="37" t="s">
         <v>924</v>
       </c>
-      <c r="C116" s="113">
+      <c r="C116" s="37">
         <v>2023</v>
       </c>
       <c r="D116" s="37" t="s">
@@ -17631,7 +17642,7 @@
       <c r="B117" s="37" t="s">
         <v>931</v>
       </c>
-      <c r="C117" s="113">
+      <c r="C117" s="37">
         <v>2025</v>
       </c>
       <c r="D117" s="37" t="s">
@@ -17755,7 +17766,7 @@
       <c r="B118" s="37" t="s">
         <v>938</v>
       </c>
-      <c r="C118" s="113">
+      <c r="C118" s="37">
         <v>2025</v>
       </c>
       <c r="D118" s="37" t="s">
@@ -17845,7 +17856,7 @@
       <c r="B119" s="37" t="s">
         <v>946</v>
       </c>
-      <c r="C119" s="113">
+      <c r="C119" s="37">
         <v>2014</v>
       </c>
       <c r="D119" s="37" t="s">
@@ -17935,7 +17946,7 @@
       <c r="B120" s="37" t="s">
         <v>953</v>
       </c>
-      <c r="C120" s="113">
+      <c r="C120" s="37">
         <v>2017</v>
       </c>
       <c r="D120" s="37" t="s">
@@ -18027,7 +18038,7 @@
       <c r="B121" s="37" t="s">
         <v>959</v>
       </c>
-      <c r="C121" s="113">
+      <c r="C121" s="37">
         <v>2020</v>
       </c>
       <c r="D121" s="37" t="s">
@@ -18115,7 +18126,7 @@
       <c r="B122" s="37" t="s">
         <v>965</v>
       </c>
-      <c r="C122" s="113">
+      <c r="C122" s="37">
         <v>2025</v>
       </c>
       <c r="D122" s="37" t="s">
@@ -18205,7 +18216,7 @@
       <c r="B123" s="37" t="s">
         <v>971</v>
       </c>
-      <c r="C123" s="113">
+      <c r="C123" s="37">
         <v>2021</v>
       </c>
       <c r="D123" s="37" t="s">
@@ -18299,7 +18310,7 @@
       <c r="B124" s="37" t="s">
         <v>979</v>
       </c>
-      <c r="C124" s="113">
+      <c r="C124" s="37">
         <v>2025</v>
       </c>
       <c r="D124" s="37" t="s">
@@ -18393,7 +18404,7 @@
       <c r="B125" s="37" t="s">
         <v>987</v>
       </c>
-      <c r="C125" s="113">
+      <c r="C125" s="37">
         <v>2007</v>
       </c>
       <c r="D125" s="37" t="s">
@@ -18483,7 +18494,7 @@
       <c r="B126" s="37" t="s">
         <v>994</v>
       </c>
-      <c r="C126" s="113">
+      <c r="C126" s="37">
         <v>2025</v>
       </c>
       <c r="D126" s="37" t="s">
@@ -18581,7 +18592,7 @@
       <c r="B127" s="37" t="s">
         <v>1001</v>
       </c>
-      <c r="C127" s="113">
+      <c r="C127" s="37">
         <v>2026</v>
       </c>
       <c r="D127" s="37" t="s">
@@ -18673,7 +18684,7 @@
       <c r="B128" s="37" t="s">
         <v>1010</v>
       </c>
-      <c r="C128" s="113">
+      <c r="C128" s="37">
         <v>2019</v>
       </c>
       <c r="D128" s="37" t="s">
@@ -18765,7 +18776,7 @@
       <c r="B129" s="37" t="s">
         <v>1014</v>
       </c>
-      <c r="C129" s="113">
+      <c r="C129" s="37">
         <v>2020</v>
       </c>
       <c r="D129" s="37" t="s">
@@ -18857,7 +18868,7 @@
       <c r="B130" s="37" t="s">
         <v>1021</v>
       </c>
-      <c r="C130" s="113">
+      <c r="C130" s="37">
         <v>2019</v>
       </c>
       <c r="D130" s="37" t="s">
@@ -18947,7 +18958,7 @@
       <c r="B131" s="37" t="s">
         <v>1028</v>
       </c>
-      <c r="C131" s="113">
+      <c r="C131" s="37">
         <v>2004</v>
       </c>
       <c r="D131" s="37" t="s">
@@ -19043,7 +19054,7 @@
       <c r="B132" s="37" t="s">
         <v>1032</v>
       </c>
-      <c r="C132" s="113">
+      <c r="C132" s="37">
         <v>2025</v>
       </c>
       <c r="D132" s="37" t="s">
@@ -19133,7 +19144,7 @@
       <c r="B133" s="37" t="s">
         <v>1040</v>
       </c>
-      <c r="C133" s="113">
+      <c r="C133" s="37">
         <v>2023</v>
       </c>
       <c r="D133" s="37" t="s">
@@ -19221,7 +19232,7 @@
       <c r="B134" s="37" t="s">
         <v>1047</v>
       </c>
-      <c r="C134" s="113">
+      <c r="C134" s="37">
         <v>2024</v>
       </c>
       <c r="D134" s="37" t="s">
@@ -19313,7 +19324,7 @@
       <c r="B135" s="37" t="s">
         <v>1055</v>
       </c>
-      <c r="C135" s="113">
+      <c r="C135" s="37">
         <v>2025</v>
       </c>
       <c r="D135" s="37" t="s">
@@ -19431,7 +19442,7 @@
       <c r="B136" s="37" t="s">
         <v>1063</v>
       </c>
-      <c r="C136" s="113">
+      <c r="C136" s="37">
         <v>2025</v>
       </c>
       <c r="D136" s="37" t="s">
@@ -19549,7 +19560,7 @@
       <c r="B137" s="37" t="s">
         <v>1070</v>
       </c>
-      <c r="C137" s="113">
+      <c r="C137" s="37">
         <v>2025</v>
       </c>
       <c r="D137" s="37" t="s">
@@ -19643,7 +19654,7 @@
       <c r="B138" s="37" t="s">
         <v>1079</v>
       </c>
-      <c r="C138" s="113">
+      <c r="C138" s="37">
         <v>2020</v>
       </c>
       <c r="D138" s="37" t="s">
@@ -19735,7 +19746,7 @@
       <c r="B139" s="37" t="s">
         <v>1086</v>
       </c>
-      <c r="C139" s="113">
+      <c r="C139" s="37">
         <v>2023</v>
       </c>
       <c r="D139" s="37" t="s">
@@ -19829,7 +19840,7 @@
       <c r="B140" s="37" t="s">
         <v>1096</v>
       </c>
-      <c r="C140" s="113">
+      <c r="C140" s="37">
         <v>2024</v>
       </c>
       <c r="D140" s="37" t="s">
@@ -19931,7 +19942,7 @@
       <c r="B141" s="37" t="s">
         <v>1103</v>
       </c>
-      <c r="C141" s="113">
+      <c r="C141" s="37">
         <v>2022</v>
       </c>
       <c r="D141" s="37" t="s">
@@ -20033,7 +20044,7 @@
       <c r="B142" s="37" t="s">
         <v>1110</v>
       </c>
-      <c r="C142" s="113">
+      <c r="C142" s="37">
         <v>2025</v>
       </c>
       <c r="D142" s="37" t="s">
@@ -20123,7 +20134,7 @@
       <c r="B143" s="37" t="s">
         <v>1115</v>
       </c>
-      <c r="C143" s="113">
+      <c r="C143" s="37">
         <v>2019</v>
       </c>
       <c r="D143" s="37" t="s">
@@ -20215,7 +20226,7 @@
       <c r="B144" s="37" t="s">
         <v>1120</v>
       </c>
-      <c r="C144" s="113">
+      <c r="C144" s="37">
         <v>2024</v>
       </c>
       <c r="D144" s="37" t="s">
@@ -20313,7 +20324,7 @@
       <c r="B145" s="37" t="s">
         <v>1126</v>
       </c>
-      <c r="C145" s="113">
+      <c r="C145" s="37">
         <v>2023</v>
       </c>
       <c r="D145" s="37" t="s">
@@ -20405,7 +20416,7 @@
       <c r="B146" s="37" t="s">
         <v>1131</v>
       </c>
-      <c r="C146" s="113">
+      <c r="C146" s="37">
         <v>2021</v>
       </c>
       <c r="D146" s="37" t="s">
@@ -20497,7 +20508,7 @@
       <c r="B147" s="37" t="s">
         <v>1137</v>
       </c>
-      <c r="C147" s="113">
+      <c r="C147" s="37">
         <v>2022</v>
       </c>
       <c r="D147" s="37" t="s">
@@ -20587,7 +20598,7 @@
       <c r="B148" s="37" t="s">
         <v>1143</v>
       </c>
-      <c r="C148" s="113">
+      <c r="C148" s="37">
         <v>2014</v>
       </c>
       <c r="D148" s="37" t="s">
@@ -20675,7 +20686,7 @@
       <c r="B149" s="37" t="s">
         <v>1150</v>
       </c>
-      <c r="C149" s="113">
+      <c r="C149" s="37">
         <v>2022</v>
       </c>
       <c r="D149" s="37" t="s">
@@ -20767,7 +20778,7 @@
       <c r="B150" s="37" t="s">
         <v>1156</v>
       </c>
-      <c r="C150" s="113">
+      <c r="C150" s="37">
         <v>2024</v>
       </c>
       <c r="D150" s="37" t="s">
@@ -20857,7 +20868,7 @@
       <c r="B151" s="37" t="s">
         <v>1162</v>
       </c>
-      <c r="C151" s="113">
+      <c r="C151" s="37">
         <v>2021</v>
       </c>
       <c r="D151" s="37" t="s">
@@ -20949,7 +20960,7 @@
       <c r="B152" s="37" t="s">
         <v>1169</v>
       </c>
-      <c r="C152" s="113">
+      <c r="C152" s="37">
         <v>2020</v>
       </c>
       <c r="D152" s="37" t="s">
@@ -21043,7 +21054,7 @@
       <c r="B153" s="37" t="s">
         <v>1176</v>
       </c>
-      <c r="C153" s="113">
+      <c r="C153" s="37">
         <v>2012</v>
       </c>
       <c r="D153" s="37" t="s">
@@ -21153,7 +21164,7 @@
       <c r="B154" s="37" t="s">
         <v>1184</v>
       </c>
-      <c r="C154" s="113">
+      <c r="C154" s="37">
         <v>2020</v>
       </c>
       <c r="D154" s="37" t="s">
@@ -21241,7 +21252,7 @@
       <c r="B155" s="37" t="s">
         <v>1190</v>
       </c>
-      <c r="C155" s="113">
+      <c r="C155" s="37">
         <v>2015</v>
       </c>
       <c r="D155" s="37" t="s">
@@ -21341,7 +21352,7 @@
       <c r="B156" s="37" t="s">
         <v>1198</v>
       </c>
-      <c r="C156" s="113">
+      <c r="C156" s="37">
         <v>2019</v>
       </c>
       <c r="D156" s="37" t="s">
@@ -21445,7 +21456,7 @@
       <c r="B157" s="37" t="s">
         <v>1204</v>
       </c>
-      <c r="C157" s="113">
+      <c r="C157" s="37">
         <v>2026</v>
       </c>
       <c r="D157" s="37" t="s">
@@ -21539,7 +21550,7 @@
       <c r="B158" s="37" t="s">
         <v>1212</v>
       </c>
-      <c r="C158" s="113">
+      <c r="C158" s="37">
         <v>2019</v>
       </c>
       <c r="D158" s="37" t="s">
@@ -21631,7 +21642,7 @@
       <c r="B159" s="37" t="s">
         <v>1219</v>
       </c>
-      <c r="C159" s="113">
+      <c r="C159" s="37">
         <v>2020</v>
       </c>
       <c r="D159" s="37" t="s">
@@ -21733,7 +21744,7 @@
       <c r="B160" s="37" t="s">
         <v>1226</v>
       </c>
-      <c r="C160" s="113">
+      <c r="C160" s="37">
         <v>2024</v>
       </c>
       <c r="D160" s="37" t="s">
@@ -21823,7 +21834,7 @@
       <c r="B161" s="37" t="s">
         <v>1233</v>
       </c>
-      <c r="C161" s="113">
+      <c r="C161" s="37">
         <v>2025</v>
       </c>
       <c r="D161" s="37" t="s">
@@ -21917,7 +21928,7 @@
       <c r="B162" s="37" t="s">
         <v>1240</v>
       </c>
-      <c r="C162" s="115">
+      <c r="C162" s="41">
         <v>2025</v>
       </c>
       <c r="D162" s="37" t="s">
@@ -22015,7 +22026,7 @@
       <c r="B163" s="37" t="s">
         <v>1246</v>
       </c>
-      <c r="C163" s="113">
+      <c r="C163" s="37">
         <v>2025</v>
       </c>
       <c r="D163" s="37" t="s">
@@ -22107,7 +22118,7 @@
       <c r="B164" s="37" t="s">
         <v>1252</v>
       </c>
-      <c r="C164" s="113">
+      <c r="C164" s="37">
         <v>2025</v>
       </c>
       <c r="D164" s="37" t="s">
@@ -22197,7 +22208,7 @@
       <c r="B165" s="37" t="s">
         <v>1260</v>
       </c>
-      <c r="C165" s="113">
+      <c r="C165" s="37">
         <v>2023</v>
       </c>
       <c r="D165" s="37" t="s">
@@ -22287,7 +22298,7 @@
       <c r="B166" s="37" t="s">
         <v>1266</v>
       </c>
-      <c r="C166" s="113">
+      <c r="C166" s="37">
         <v>1975</v>
       </c>
       <c r="D166" s="37" t="s">
@@ -22377,7 +22388,7 @@
       <c r="B167" s="37" t="s">
         <v>1273</v>
       </c>
-      <c r="C167" s="113">
+      <c r="C167" s="37">
         <v>2024</v>
       </c>
       <c r="D167" s="37" t="s">
@@ -22473,7 +22484,7 @@
       <c r="B168" s="63" t="s">
         <v>1276</v>
       </c>
-      <c r="C168" s="116">
+      <c r="C168" s="63">
         <v>2016</v>
       </c>
       <c r="D168" s="63" t="s">
@@ -22571,7 +22582,7 @@
       <c r="B169" s="63" t="s">
         <v>1286</v>
       </c>
-      <c r="C169" s="116">
+      <c r="C169" s="63">
         <v>2019</v>
       </c>
       <c r="D169" s="63" t="s">
@@ -22661,7 +22672,7 @@
       <c r="B170" s="63" t="s">
         <v>1293</v>
       </c>
-      <c r="C170" s="116">
+      <c r="C170" s="63">
         <v>2024</v>
       </c>
       <c r="D170" s="63" t="s">
@@ -22779,7 +22790,7 @@
       <c r="B171" s="37" t="s">
         <v>1298</v>
       </c>
-      <c r="C171" s="117">
+      <c r="C171">
         <v>2022</v>
       </c>
       <c r="D171" s="3" t="s">
@@ -22844,7 +22855,7 @@
       <c r="B172" s="3" t="s">
         <v>1303</v>
       </c>
-      <c r="C172" s="117">
+      <c r="C172">
         <v>2023</v>
       </c>
       <c r="D172" s="3" t="s">
@@ -22906,7 +22917,7 @@
       <c r="B173" s="3" t="s">
         <v>1309</v>
       </c>
-      <c r="C173" s="117">
+      <c r="C173">
         <v>2025</v>
       </c>
       <c r="D173" s="10" t="s">
@@ -22983,7 +22994,7 @@
       <c r="B174" s="3" t="s">
         <v>1314</v>
       </c>
-      <c r="C174" s="117">
+      <c r="C174">
         <v>2024</v>
       </c>
       <c r="D174" s="3" t="s">
@@ -23039,7 +23050,7 @@
       <c r="B175" s="3" t="s">
         <v>1319</v>
       </c>
-      <c r="C175" s="117">
+      <c r="C175">
         <v>2023</v>
       </c>
       <c r="D175" s="10" t="s">
@@ -23096,7 +23107,7 @@
       <c r="B176" s="37" t="s">
         <v>1351</v>
       </c>
-      <c r="C176" s="118">
+      <c r="C176" s="83">
         <v>2022</v>
       </c>
       <c r="D176" s="87" t="s">
@@ -23196,7 +23207,7 @@
       <c r="B177" s="3" t="s">
         <v>1364</v>
       </c>
-      <c r="C177" s="118">
+      <c r="C177" s="83">
         <v>2023</v>
       </c>
       <c r="D177" s="3" t="s">
@@ -23286,7 +23297,7 @@
       <c r="B178" s="3" t="s">
         <v>1372</v>
       </c>
-      <c r="C178" s="118">
+      <c r="C178" s="83">
         <v>2024</v>
       </c>
       <c r="D178" s="3" t="s">
@@ -23376,7 +23387,7 @@
       <c r="B179" s="3" t="s">
         <v>1376</v>
       </c>
-      <c r="C179" s="118">
+      <c r="C179" s="83">
         <v>2024</v>
       </c>
       <c r="D179" s="3" t="s">
@@ -23462,7 +23473,7 @@
       <c r="B180" s="3" t="s">
         <v>1381</v>
       </c>
-      <c r="C180" s="118">
+      <c r="C180" s="83">
         <v>2026</v>
       </c>
       <c r="D180" s="3" t="s">
@@ -23552,7 +23563,7 @@
       <c r="B181" s="3" t="s">
         <v>1391</v>
       </c>
-      <c r="C181" s="118">
+      <c r="C181" s="83">
         <v>2026</v>
       </c>
       <c r="D181" s="3" t="s">
@@ -23642,7 +23653,7 @@
       <c r="B182" s="3" t="s">
         <v>1396</v>
       </c>
-      <c r="C182" s="118">
+      <c r="C182" s="83">
         <v>2023</v>
       </c>
       <c r="D182" s="3" t="s">
@@ -23758,7 +23769,7 @@
       <c r="B183" s="3" t="s">
         <v>1403</v>
       </c>
-      <c r="C183" s="118">
+      <c r="C183" s="83">
         <v>2021</v>
       </c>
       <c r="D183" s="3" t="s">
@@ -23870,7 +23881,7 @@
       <c r="B184" s="3" t="s">
         <v>1415</v>
       </c>
-      <c r="C184" s="118">
+      <c r="C184" s="83">
         <v>2023</v>
       </c>
       <c r="D184" s="3" t="s">
@@ -23960,7 +23971,7 @@
       <c r="B185" s="3" t="s">
         <v>1414</v>
       </c>
-      <c r="C185" s="118">
+      <c r="C185" s="83">
         <v>2026</v>
       </c>
       <c r="D185" s="3" t="s">
@@ -24056,7 +24067,7 @@
       <c r="B186" t="s">
         <v>1437</v>
       </c>
-      <c r="C186" s="117">
+      <c r="C186">
         <v>2025</v>
       </c>
       <c r="D186" t="s">
@@ -24175,7 +24186,7 @@
       <c r="B187" t="s">
         <v>1436</v>
       </c>
-      <c r="C187" s="117">
+      <c r="C187">
         <v>2026</v>
       </c>
       <c r="D187" t="s">
@@ -24278,7 +24289,7 @@
       <c r="B188" s="3" t="s">
         <v>1439</v>
       </c>
-      <c r="C188" s="118">
+      <c r="C188" s="83">
         <v>2026</v>
       </c>
       <c r="D188" s="3" t="s">
@@ -24362,8 +24373,104 @@
       </c>
     </row>
     <row r="189" spans="1:54" ht="14.3" customHeight="1">
-      <c r="A189" s="70"/>
-      <c r="AW189" s="10"/>
+      <c r="A189" s="70">
+        <v>188</v>
+      </c>
+      <c r="B189" s="3" t="s">
+        <v>1444</v>
+      </c>
+      <c r="C189" s="114">
+        <v>2026</v>
+      </c>
+      <c r="D189" s="3" t="s">
+        <v>1445</v>
+      </c>
+      <c r="E189" s="89" t="s">
+        <v>1446</v>
+      </c>
+      <c r="F189" s="68" t="s">
+        <v>117</v>
+      </c>
+      <c r="G189" s="90" t="s">
+        <v>117</v>
+      </c>
+      <c r="H189" s="49" t="s">
+        <v>329</v>
+      </c>
+      <c r="I189" s="77" t="s">
+        <v>240</v>
+      </c>
+      <c r="J189" s="81"/>
+      <c r="K189" s="91" t="s">
+        <v>1447</v>
+      </c>
+      <c r="L189" s="83" t="s">
+        <v>1399</v>
+      </c>
+      <c r="M189" s="49" t="s">
+        <v>107</v>
+      </c>
+      <c r="N189" s="82"/>
+      <c r="O189" s="82"/>
+      <c r="P189" s="82">
+        <v>3</v>
+      </c>
+      <c r="Q189" s="82"/>
+      <c r="R189" s="82">
+        <v>3</v>
+      </c>
+      <c r="S189" s="82">
+        <v>3</v>
+      </c>
+      <c r="T189" s="82">
+        <v>3</v>
+      </c>
+      <c r="U189" s="82">
+        <v>3</v>
+      </c>
+      <c r="V189" s="82"/>
+      <c r="W189" s="82"/>
+      <c r="X189" s="82"/>
+      <c r="Y189" s="82">
+        <v>3</v>
+      </c>
+      <c r="Z189" s="82"/>
+      <c r="AA189" s="82"/>
+      <c r="AB189" s="82"/>
+      <c r="AC189" s="82"/>
+      <c r="AD189" s="82"/>
+      <c r="AE189" s="82"/>
+      <c r="AF189" s="82"/>
+      <c r="AG189" s="82"/>
+      <c r="AH189" s="82"/>
+      <c r="AI189" s="82"/>
+      <c r="AJ189" s="82"/>
+      <c r="AK189" s="82"/>
+      <c r="AL189" s="82"/>
+      <c r="AM189" s="82"/>
+      <c r="AN189" s="82"/>
+      <c r="AO189" s="67"/>
+      <c r="AP189" s="82"/>
+      <c r="AQ189" s="82"/>
+      <c r="AR189" s="82"/>
+      <c r="AS189" s="82"/>
+      <c r="AT189" s="67"/>
+      <c r="AU189" s="82"/>
+      <c r="AV189" s="82"/>
+      <c r="AW189" s="10" t="s">
+        <v>1450</v>
+      </c>
+      <c r="AX189" s="83"/>
+      <c r="AY189" s="83"/>
+      <c r="AZ189" s="10" t="s">
+        <v>1393</v>
+      </c>
+      <c r="BA189" s="45" t="s">
+        <v>1449</v>
+      </c>
+      <c r="BB189" s="10" t="s">
+        <v>1448</v>
+      </c>
     </row>
     <row r="190" spans="1:54" ht="14.3" customHeight="1">
       <c r="A190" s="70"/>
@@ -27680,16 +27787,16 @@
     <row r="1018" spans="1:49" ht="14.3" customHeight="1"/>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="Q1:AD1"/>
+    <mergeCell ref="AE1:AF1"/>
     <mergeCell ref="AG1:AJ1"/>
     <mergeCell ref="AN1:AO1"/>
     <mergeCell ref="AP1:AQ1"/>
     <mergeCell ref="AR1:AU1"/>
     <mergeCell ref="AZ1:BB1"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="Q1:AD1"/>
-    <mergeCell ref="AE1:AF1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="E144" r:id="rId1" xr:uid="{A81C656A-0A99-4267-9649-0EEFD2B27222}"/>
@@ -27702,10 +27809,11 @@
     <hyperlink ref="E184" r:id="rId8" display="https://doi.org/10.1016/j.ocecoaman.2023.106771" xr:uid="{544CA07B-2E2A-4DBC-9CC6-55FE9D10C148}"/>
     <hyperlink ref="E185" r:id="rId9" xr:uid="{9D95C0B9-0AF7-4B80-8A81-ABCD934682EF}"/>
     <hyperlink ref="E188" r:id="rId10" tooltip="DOI URL" xr:uid="{71E22F72-0CF3-4154-834D-5AA603563583}"/>
+    <hyperlink ref="E189" r:id="rId11" xr:uid="{C96102E8-A232-4FB7-86C2-1DF66DEBB549}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId11"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>